<commit_message>
changed variable names to add com_ as prep for merge
</commit_message>
<xml_diff>
--- a/data/final_datasets/feature_dictionary_commercial.xlsx
+++ b/data/final_datasets/feature_dictionary_commercial.xlsx
@@ -561,7 +561,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>median_age_level_2026</t>
+          <t>com_median_age_level_2026</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -601,7 +601,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>median_age_slope</t>
+          <t>com_median_age_slope</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -641,7 +641,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>median_age_r2</t>
+          <t>com_median_age_r2</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -681,7 +681,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>share_max_1y_level_2026</t>
+          <t>com_share_max_1y_level_2026</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -721,7 +721,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>share_max_1y_slope</t>
+          <t>com_share_max_1y_slope</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -761,7 +761,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>share_max_1y_r2</t>
+          <t>com_share_max_1y_r2</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -801,7 +801,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>share_max_2y_level_2026</t>
+          <t>com_share_max_2y_level_2026</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -841,7 +841,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>share_max_2y_slope</t>
+          <t>com_share_max_2y_slope</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -881,7 +881,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>share_max_2y_r2</t>
+          <t>com_share_max_2y_r2</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -921,7 +921,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>share_max_5y_level_2026</t>
+          <t>com_share_max_5y_level_2026</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -961,7 +961,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>share_max_5y_slope</t>
+          <t>com_share_max_5y_slope</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1001,7 +1001,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>share_max_5y_r2</t>
+          <t>com_share_max_5y_r2</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1041,7 +1041,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>share_min_20y_level_2026</t>
+          <t>com_share_min_20y_level_2026</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1081,7 +1081,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>share_min_20y_slope</t>
+          <t>com_share_min_20y_slope</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1121,7 +1121,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>share_min_20y_r2</t>
+          <t>com_share_min_20y_r2</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1161,7 +1161,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>share_min_30y_level_2026</t>
+          <t>com_share_min_30y_level_2026</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1201,7 +1201,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>share_min_30y_slope</t>
+          <t>com_share_min_30y_slope</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>share_min_30y_r2</t>
+          <t>com_share_min_30y_r2</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1281,7 +1281,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>share_min_40y_level_2026</t>
+          <t>com_share_min_40y_level_2026</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1321,7 +1321,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>share_min_40y_slope</t>
+          <t>com_share_min_40y_slope</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1361,7 +1361,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>share_min_40y_r2</t>
+          <t>com_share_min_40y_r2</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1401,7 +1401,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>share_solo_level_2026</t>
+          <t>com_share_solo_level_2026</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -1441,7 +1441,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>share_solo_slope</t>
+          <t>com_share_solo_slope</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1481,7 +1481,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>share_solo_r2</t>
+          <t>com_share_solo_r2</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -1521,7 +1521,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>share_1_9_level_2026</t>
+          <t>com_share_1_9_level_2026</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1561,7 +1561,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>share_1_9_slope</t>
+          <t>com_share_1_9_slope</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -1601,7 +1601,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>share_1_9_r2</t>
+          <t>com_share_1_9_r2</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1641,7 +1641,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>share_10plus_level_2026</t>
+          <t>com_share_10plus_level_2026</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1681,7 +1681,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>share_10plus_slope</t>
+          <t>com_share_10plus_slope</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1721,7 +1721,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>share_10plus_r2</t>
+          <t>com_share_10plus_r2</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -1761,7 +1761,7 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>gastro_share_level_2026</t>
+          <t>com_gastro_share_level_2026</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1801,7 +1801,7 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>gastro_share_slope</t>
+          <t>com_gastro_share_slope</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -1841,7 +1841,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>gastro_share_r2</t>
+          <t>com_gastro_share_r2</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1881,7 +1881,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>upscale_share_level_2026</t>
+          <t>com_upscale_share_level_2026</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -1921,7 +1921,7 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>upscale_share_slope</t>
+          <t>com_upscale_share_slope</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -1961,7 +1961,7 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>upscale_share_r2</t>
+          <t>com_upscale_share_r2</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
@@ -2001,7 +2001,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>gastro_quotient_bezirk_level_2026</t>
+          <t>com_gastro_quotient_bezirk_level_2026</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -2041,7 +2041,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>gastro_quotient_bezirk_slope</t>
+          <t>com_gastro_quotient_bezirk_slope</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -2081,7 +2081,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>gastro_quotient_bezirk_r2</t>
+          <t>com_gastro_quotient_bezirk_r2</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -2121,7 +2121,7 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>gastro_quotient_berlin_level_2026</t>
+          <t>com_gastro_quotient_berlin_level_2026</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -2161,7 +2161,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>gastro_quotient_berlin_slope</t>
+          <t>com_gastro_quotient_berlin_slope</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -2201,7 +2201,7 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>gastro_quotient_berlin_r2</t>
+          <t>com_gastro_quotient_berlin_r2</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -2241,7 +2241,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>upscale_quotient_bezirk_level_2026</t>
+          <t>com_upscale_quotient_bezirk_level_2026</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -2281,7 +2281,7 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>upscale_quotient_bezirk_slope</t>
+          <t>com_upscale_quotient_bezirk_slope</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
@@ -2321,7 +2321,7 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>upscale_quotient_bezirk_r2</t>
+          <t>com_upscale_quotient_bezirk_r2</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -2361,7 +2361,7 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>upscale_quotient_berlin_level_2026</t>
+          <t>com_upscale_quotient_berlin_level_2026</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
@@ -2401,7 +2401,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>upscale_quotient_berlin_slope</t>
+          <t>com_upscale_quotient_berlin_slope</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -2441,7 +2441,7 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>upscale_quotient_berlin_r2</t>
+          <t>com_upscale_quotient_berlin_r2</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
@@ -2481,7 +2481,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>tourism_share_level_2026</t>
+          <t>com_tourism_share_level_2026</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -2521,7 +2521,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>tourism_share_slope</t>
+          <t>com_tourism_share_slope</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -2561,7 +2561,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>tourism_share_r2</t>
+          <t>com_tourism_share_r2</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
@@ -2601,7 +2601,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>tourism_quotient_bezirk_level_2026</t>
+          <t>com_tourism_quotient_bezirk_level_2026</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -2641,7 +2641,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>tourism_quotient_bezirk_slope</t>
+          <t>com_tourism_quotient_bezirk_slope</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
@@ -2681,7 +2681,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>tourism_quotient_bezirk_r2</t>
+          <t>com_tourism_quotient_bezirk_r2</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
@@ -2721,7 +2721,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>tourism_quotient_berlin_level_2026</t>
+          <t>com_tourism_quotient_berlin_level_2026</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
@@ -2761,7 +2761,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>tourism_quotient_berlin_slope</t>
+          <t>com_tourism_quotient_berlin_slope</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -2801,7 +2801,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>tourism_quotient_berlin_r2</t>
+          <t>com_tourism_quotient_berlin_r2</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
@@ -2841,7 +2841,7 @@
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>n_gastro</t>
+          <t>com_n_gastro</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -2881,7 +2881,7 @@
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>n_upscale</t>
+          <t>com_n_upscale</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -2921,7 +2921,7 @@
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>has_gastro_structure</t>
+          <t>com_has_gastro_structure</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">

</xml_diff>